<commit_message>
update bill page 6486819279
</commit_message>
<xml_diff>
--- a/bills/huixinjiqiren/6486819279/7245cad451d2a4c1ec431882c82a535377c2a9e9001db1872bda3e78a0d6f36f/bill-2026-09-30.xlsx
+++ b/bills/huixinjiqiren/6486819279/7245cad451d2a4c1ec431882c82a535377c2a9e9001db1872bda3e78a0d6f36f/bill-2026-09-30.xlsx
@@ -90,12 +90,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>111.11</t>
+          <t>125</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -227,7 +227,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>111.11</t>
+          <t>125</t>
         </is>
       </c>
     </row>
@@ -251,7 +251,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>111.11</t>
+          <t>125</t>
         </is>
       </c>
     </row>

</xml_diff>